<commit_message>
ultimas melhorias na estrutura do sistema, inclusão de meta de abril no banco de dados
</commit_message>
<xml_diff>
--- a/metas.xlsx
+++ b/metas.xlsx
@@ -152,7 +152,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultColWidth="14.4375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.4453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -164,251 +164,247 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="n">
-        <v>46082</v>
+        <v>46113</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>4694.97776</v>
+        <v>2951.8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
-        <v>46083</v>
+        <v>46114</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2600.96311538462</v>
+        <v>2871.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
-        <v>46084</v>
+        <v>46115</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>2691.10346153846</v>
+        <v>2948.3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="n">
-        <v>46085</v>
+        <v>46116</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>3000.2225</v>
+        <v>4705.97</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="n">
-        <v>46086</v>
+        <v>46117</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>3049.44030769231</v>
+        <v>4690.86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="n">
-        <v>46087</v>
+        <v>46118</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3011.866</v>
+        <v>2460.24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="n">
-        <v>46088</v>
+        <v>46119</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>4793.87107692308</v>
+        <v>2676.45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="n">
-        <v>46089</v>
+        <v>46120</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>4694.97776</v>
+        <v>2951.8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="n">
-        <v>46090</v>
+        <v>46121</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>2600.96311538462</v>
+        <v>2871.2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="n">
-        <v>46091</v>
+        <v>46122</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>2691.10346153846</v>
+        <v>2948.3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="n">
-        <v>46092</v>
+        <v>46123</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>3000.2225</v>
+        <v>4705.97</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="n">
-        <v>46093</v>
+        <v>46124</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>3049.44030769231</v>
+        <v>4690.86</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="n">
-        <v>46094</v>
+        <v>46125</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>3011.866</v>
+        <v>2460.24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="n">
-        <v>46095</v>
+        <v>46126</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>4793.87107692308</v>
+        <v>2676.45</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="n">
-        <v>46096</v>
+        <v>46127</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>4694.97776</v>
+        <v>2951.8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="n">
-        <v>46097</v>
+        <v>46128</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2600.96311538462</v>
+        <v>2871.2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="n">
-        <v>46098</v>
+        <v>46129</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>2691.10346153846</v>
+        <v>2948.3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="n">
-        <v>46099</v>
+        <v>46130</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>3000.2225</v>
+        <v>4705.97</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="n">
-        <v>46100</v>
+        <v>46131</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>3049.44030769231</v>
+        <v>4690.86</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="n">
-        <v>46101</v>
+        <v>46132</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>3011.866</v>
+        <v>2460.24</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="n">
-        <v>46102</v>
+        <v>46133</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>4793.87107692308</v>
+        <v>2676.45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="n">
-        <v>46103</v>
+        <v>46134</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>4694.97776</v>
+        <v>2951.8</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="n">
-        <v>46104</v>
+        <v>46135</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>2600.96311538462</v>
+        <v>2871.2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="n">
-        <v>46105</v>
+        <v>46136</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>2691.10346153846</v>
+        <v>2948.3</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="n">
-        <v>46106</v>
+        <v>46137</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>3000.2225</v>
+        <v>4705.97</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="n">
-        <v>46107</v>
+        <v>46138</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>3049.44030769231</v>
+        <v>4690.86</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="n">
-        <v>46108</v>
+        <v>46139</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>3011.866</v>
+        <v>2460.24</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="n">
-        <v>46109</v>
+        <v>46140</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>4793.87107692308</v>
+        <v>2676.45</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="n">
-        <v>46110</v>
+        <v>46141</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>4694.97776</v>
+        <v>2951.8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="n">
-        <v>46111</v>
+        <v>46142</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>2600.96311538462</v>
+        <v>2871.2</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="n">
-        <v>46112</v>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>2691.10346153846</v>
-      </c>
+      <c r="A32" s="3"/>
+      <c r="B32" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>